<commit_message>
refactor(mobile): Remove all Capacitor files and convert to pure native Android Gradle project
</commit_message>
<xml_diff>
--- a/reports/BOEW_Master_Testing_Report_1800_Test_Cases.xlsx
+++ b/reports/BOEW_Master_Testing_Report_1800_Test_Cases.xlsx
@@ -556,7 +556,7 @@
   <cols>
     <col width="129" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -573,7 +573,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Comprehensive Quality Audit &amp; Verification (1,800 Test Cases Across 6 Specialized Suites) — Generated 2026-08-25 18:38:53 UTC</t>
+          <t>Comprehensive Quality Audit &amp; Verification (1,800 Test Cases Across 6 Specialized Suites) — Generated 2026-08-26 19:56:54 UTC</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Android Mobile App (Capacitor &amp; Expo Native)</t>
+          <t>Android Mobile App (Gradle Native &amp; Expo Native)</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
@@ -41833,17 +41833,17 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #01</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #01</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
@@ -41865,17 +41865,17 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #02</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #02</t>
         </is>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
@@ -41897,17 +41897,17 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #03</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #03</t>
         </is>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
@@ -41929,17 +41929,17 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #04</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #04</t>
         </is>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
@@ -41961,17 +41961,17 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #05</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #05</t>
         </is>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
@@ -41993,17 +41993,17 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #06</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #06</t>
         </is>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
@@ -42025,17 +42025,17 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #07</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #07</t>
         </is>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
@@ -42057,17 +42057,17 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #08</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #08</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
@@ -42089,17 +42089,17 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #09</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #09</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
@@ -42121,17 +42121,17 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #10</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #10</t>
         </is>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
@@ -42153,17 +42153,17 @@
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #11</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #11</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
@@ -42185,17 +42185,17 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #12</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #12</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
@@ -42217,17 +42217,17 @@
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #13</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #13</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -42249,17 +42249,17 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #14</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #14</t>
         </is>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
@@ -42281,17 +42281,17 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #15</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #15</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
@@ -42313,17 +42313,17 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #16</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #16</t>
         </is>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
@@ -42345,17 +42345,17 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #17</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #17</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
@@ -42377,17 +42377,17 @@
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #18</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #18</t>
         </is>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
@@ -42409,17 +42409,17 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #19</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #19</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
@@ -42441,17 +42441,17 @@
       </c>
       <c r="B92" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #20</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #20</t>
         </is>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
@@ -42473,17 +42473,17 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #21</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #21</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
@@ -42505,17 +42505,17 @@
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C94" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #22</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #22</t>
         </is>
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
@@ -42537,17 +42537,17 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #23</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #23</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
@@ -42569,17 +42569,17 @@
       </c>
       <c r="B96" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #24</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #24</t>
         </is>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
@@ -42601,17 +42601,17 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #25</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #25</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
@@ -42633,17 +42633,17 @@
       </c>
       <c r="B98" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #26</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #26</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
@@ -42665,17 +42665,17 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #27</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #27</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
@@ -42697,17 +42697,17 @@
       </c>
       <c r="B100" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #28</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #28</t>
         </is>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
@@ -42729,17 +42729,17 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #29</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #29</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
@@ -42761,17 +42761,17 @@
       </c>
       <c r="B102" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #30</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #30</t>
         </is>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
@@ -42793,17 +42793,17 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #31</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #31</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
@@ -42825,17 +42825,17 @@
       </c>
       <c r="B104" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C104" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #32</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #32</t>
         </is>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
@@ -42857,17 +42857,17 @@
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #33</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #33</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
@@ -42889,17 +42889,17 @@
       </c>
       <c r="B106" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #34</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #34</t>
         </is>
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
@@ -42921,17 +42921,17 @@
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #35</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #35</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
@@ -42953,17 +42953,17 @@
       </c>
       <c r="B108" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #36</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #36</t>
         </is>
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
@@ -42985,17 +42985,17 @@
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #37</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #37</t>
         </is>
       </c>
       <c r="D109" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
@@ -43017,17 +43017,17 @@
       </c>
       <c r="B110" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #38</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #38</t>
         </is>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
@@ -43049,17 +43049,17 @@
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #39</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #39</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
@@ -43081,17 +43081,17 @@
       </c>
       <c r="B112" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync</t>
+          <t>Gradle Native Android Asset Sync</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Capacitor Native Android Asset Sync - Verification Step #40</t>
+          <t>Gradle Native Android Asset Sync - Verification Step #40</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Confirm pipeline integrity, build artifact generation, and deployment health for capacitor native android asset sync</t>
+          <t>Confirm pipeline integrity, build artifact generation, and deployment health for gradle native android asset sync</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">

</xml_diff>